<commit_message>
Firebase bagimliligini kaldir MySQL JWT mimarisine gec
</commit_message>
<xml_diff>
--- a/database/canias-data-entry-template.xlsx
+++ b/database/canias-data-entry-template.xlsx
@@ -1365,7 +1365,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Firebase UID</t>
+          <t>Şifre Hash (Sistem)</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>firebase_uid</t>
+          <t>password_hash</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Firebase Auth hesabı oluşturulduktan sonra yazılır; ilk aşamada boş olabilir</t>
+          <t>Elle yazılmaz; uygulama bcrypt hash üretir</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">

</xml_diff>